<commit_message>
Per visite gesynchroniseerd met de handmatige aanpassingen in Per nummer
Per nummer is de leidende map (alle inhoudelijke correcties zijn daar
doorgevoerd); alle 102 betrokken bestanden in Per visite bijgewerkt naar
diezelfde inhoud. 145 documenten geverifieerd, geen fouten.
</commit_message>
<xml_diff>
--- a/(e)CRF/Per nummer/00_Patienten-identificatielijst.xlsx
+++ b/(e)CRF/Per nummer/00_Patienten-identificatielijst.xlsx
@@ -5002,7 +5002,7 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B7 A1:C5 A6 C6 E6">
+  <conditionalFormatting sqref="A1:C5 A6 C6 E6 A7:B7">
     <cfRule type="timePeriod" dxfId="21" priority="1" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
@@ -6822,24 +6822,24 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A6 C6 E6">
+    <cfRule type="timePeriod" dxfId="19" priority="1" timePeriod="nextWeek">
+      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A7:B7">
-    <cfRule type="timePeriod" dxfId="19" priority="2" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="18" priority="2" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:C5">
-    <cfRule type="timePeriod" dxfId="18" priority="4" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="17" priority="4" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:E2">
-    <cfRule type="timePeriod" dxfId="17" priority="5" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="16" priority="5" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(D1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(D1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6 C6 E6">
-    <cfRule type="timePeriod" dxfId="4" priority="1" timePeriod="nextWeek">
-      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8652,24 +8652,24 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A6 C6 E6">
+    <cfRule type="timePeriod" dxfId="15" priority="1" timePeriod="nextWeek">
+      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A7:B7">
-    <cfRule type="timePeriod" dxfId="16" priority="2" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="14" priority="2" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:C5">
-    <cfRule type="timePeriod" dxfId="15" priority="4" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="13" priority="4" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:E2">
-    <cfRule type="timePeriod" dxfId="14" priority="5" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="12" priority="5" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(D1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(D1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6 C6 E6">
-    <cfRule type="timePeriod" dxfId="3" priority="1" timePeriod="nextWeek">
-      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10482,24 +10482,24 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A6 C6 E6">
+    <cfRule type="timePeriod" dxfId="11" priority="1" timePeriod="nextWeek">
+      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A7:B7">
-    <cfRule type="timePeriod" dxfId="13" priority="2" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="10" priority="2" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:C5">
-    <cfRule type="timePeriod" dxfId="12" priority="4" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="9" priority="4" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:E2">
-    <cfRule type="timePeriod" dxfId="11" priority="5" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="8" priority="5" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(D1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(D1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6 C6 E6">
-    <cfRule type="timePeriod" dxfId="2" priority="1" timePeriod="nextWeek">
-      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12312,24 +12312,24 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A6 C6 E6">
+    <cfRule type="timePeriod" dxfId="7" priority="1" timePeriod="nextWeek">
+      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A7:B7">
-    <cfRule type="timePeriod" dxfId="10" priority="2" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="6" priority="2" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:C5">
-    <cfRule type="timePeriod" dxfId="9" priority="4" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="5" priority="4" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:E2">
-    <cfRule type="timePeriod" dxfId="8" priority="5" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="4" priority="5" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(D1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(D1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6 C6 E6">
-    <cfRule type="timePeriod" dxfId="1" priority="1" timePeriod="nextWeek">
-      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14145,24 +14145,24 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A6 C6 E6">
+    <cfRule type="timePeriod" dxfId="3" priority="1" timePeriod="nextWeek">
+      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A7:B7">
-    <cfRule type="timePeriod" dxfId="7" priority="2" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="2" priority="2" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:C5">
-    <cfRule type="timePeriod" dxfId="6" priority="4" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="1" priority="4" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:E2">
-    <cfRule type="timePeriod" dxfId="5" priority="5" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="0" priority="5" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(D1,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(D1,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6 C6 E6">
-    <cfRule type="timePeriod" dxfId="0" priority="1" timePeriod="nextWeek">
-      <formula>AND(ROUNDDOWN(A6,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A6,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14245,21 +14245,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F1B33D7B57FFEC4BB77B5001C5B93838" ma:contentTypeVersion="6" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="59579db12405a868ad0e92c5e4f74ae1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f44e6bd5-09db-4117-8b15-adf399208dc6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="98cf673e6ff17a9b7a889e3f7df574b2" ns2:_="">
     <xsd:import namespace="f44e6bd5-09db-4117-8b15-adf399208dc6"/>
@@ -14415,24 +14400,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BDCF903-BA31-4DB0-B467-C3CC1B28989E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88182F73-E0BA-40D2-A01B-FE2F1A72F50B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F72EF480-3E9C-466F-BA1A-D34CBC3C9DDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14448,4 +14431,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88182F73-E0BA-40D2-A01B-FE2F1A72F50B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BDCF903-BA31-4DB0-B467-C3CC1B28989E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>